<commit_message>
Add Q1-Q4 quarter filtering, master importer, and UI consistency fixes
- Add clickable Q1-Q4 quarter toggle buttons on Dashboard and Stores pages
- All scores now filter by selected quarter instead of showing latest
- Rename BI Dashboard button to Power BI with chart icon
- Add import_master.py for robust Excel data ingestion with adaptive parsing
- Fix risk column truncation (String(20) -> Text) for Postgres
- Update StoreAuditScores to use quarterly scores from API
- Connect all frontend pages to backend API (no more mock data)
- Add .env.example and dummy Excel templates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/uploads/store_scores.xlsx
+++ b/backend/uploads/store_scores.xlsx
@@ -17,13 +17,22 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,332 +426,341 @@
   </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Store ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Store Code</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ST001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>RC-MUM-001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="D2" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ST002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>RC-DEL-001</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ST003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>RC-BLR-001</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="F4" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="F2" t="n">
-        <v>70.90000000000001</v>
-      </c>
-      <c r="G2" t="n">
-        <v>73.3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ST002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RC-DEL-001</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="G4" s="2" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ST004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>RC-DEL-002</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="E3" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="F3" t="n">
-        <v>66.59999999999999</v>
-      </c>
-      <c r="G3" t="n">
-        <v>67.8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ST003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>RC-BLR-001</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="D5" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ST005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>RC-PUN-001</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="F4" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>88.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ST004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>RC-DEL-002</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="D6" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ST006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>RC-CHD-001</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>59.2</v>
-      </c>
-      <c r="E5" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="F5" t="n">
-        <v>57</v>
-      </c>
-      <c r="G5" t="n">
-        <v>57.7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ST005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>RC-PUN-001</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="D7" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ST007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>RC-NAG-001</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>71</v>
-      </c>
-      <c r="E6" t="n">
-        <v>76.3</v>
-      </c>
-      <c r="F6" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="G6" t="n">
-        <v>68.90000000000001</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ST006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>RC-CHD-001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="D8" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ST008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>RC-DDN-001</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="F7" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>66.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ST007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>RC-NAG-001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Operating</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>85.59999999999999</v>
-      </c>
-      <c r="E8" t="n">
-        <v>89.2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>86.90000000000001</v>
-      </c>
-      <c r="G8" t="n">
-        <v>84.2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ST008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>RC-DDN-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Operating</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>69.2</v>
-      </c>
-      <c r="E9" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="F9" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>67.3</v>
+      <c r="D9" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ST009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>RC-KOL-001</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Dehired</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>79.5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="F10" t="n">
-        <v>77.7</v>
-      </c>
-      <c r="G10" t="n">
-        <v>76</v>
+      <c r="D10" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ST010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>RC-JAI-001</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Dehired</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>73.09999999999999</v>
-      </c>
-      <c r="E11" t="n">
-        <v>72.09999999999999</v>
-      </c>
-      <c r="F11" t="n">
-        <v>72.3</v>
-      </c>
-      <c r="G11" t="n">
-        <v>75.5</v>
+      <c r="D11" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>